<commit_message>
put color column back in species table
</commit_message>
<xml_diff>
--- a/NWspecies060222.xlsx
+++ b/NWspecies060222.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0f4fad9919cbe5b/Neighbourwoods/NWAnalytics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="8_{DD247510-64D4-4C56-90AC-C75474531547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{572C582A-EEF0-4D97-BB9E-96A60D4F4A3F}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="8_{DD247510-64D4-4C56-90AC-C75474531547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D35ADC4-AD9E-4400-91C2-0CA214A1A8D0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19616" uniqueCount="2268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19916" uniqueCount="2269">
   <si>
     <t>ID</t>
   </si>
@@ -6856,6 +6856,9 @@
   </si>
   <si>
     <t>Nanny Berry</t>
+  </si>
+  <si>
+    <t>pink</t>
   </si>
 </sst>
 </file>
@@ -7771,7 +7774,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O301"/>
+  <dimension ref="A1:P301"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.140625" customWidth="1"/>
@@ -7787,7 +7790,7 @@
     <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="7" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="7" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -7833,8 +7836,11 @@
       <c r="O1" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P1" s="7" t="s">
+        <v>2107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7880,8 +7886,11 @@
       <c r="O2">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P2" t="s">
+        <v>2108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7927,8 +7936,11 @@
       <c r="O3">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P3" t="s">
+        <v>2109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7971,8 +7983,11 @@
       <c r="O4">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P4" t="s">
+        <v>2111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -8018,8 +8033,11 @@
       <c r="O5">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P5" t="s">
+        <v>2112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>318</v>
       </c>
@@ -8059,8 +8077,11 @@
       <c r="M6" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P6" t="s">
+        <v>2121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -8100,8 +8121,11 @@
       <c r="M7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P7" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -8147,8 +8171,11 @@
       <c r="O8">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P8" t="s">
+        <v>2142</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -8188,8 +8215,11 @@
       <c r="M9" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P9" t="s">
+        <v>2144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>282</v>
       </c>
@@ -8229,8 +8259,11 @@
       <c r="M10" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P10" t="s">
+        <v>2146</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -8276,8 +8309,11 @@
       <c r="O11">
         <v>0.84</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P11" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -8323,8 +8359,11 @@
       <c r="O12">
         <v>0.84</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P12" t="s">
+        <v>2152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -8370,8 +8409,11 @@
       <c r="O13">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P13" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -8417,8 +8459,11 @@
       <c r="O14">
         <v>0.83</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P14" t="s">
+        <v>2156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -8464,8 +8509,11 @@
       <c r="O15">
         <v>0.84</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P15" t="s">
+        <v>2161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -8508,8 +8556,11 @@
       <c r="O16">
         <v>0.84</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P16" t="s">
+        <v>2163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -8555,8 +8606,11 @@
       <c r="O17">
         <v>0.84</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P17" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -8602,8 +8656,11 @@
       <c r="O18">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P18" t="s">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -8649,8 +8706,11 @@
       <c r="O19">
         <v>0.74</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P19" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -8696,8 +8756,11 @@
       <c r="O20">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P20" t="s">
+        <v>2184</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -8743,8 +8806,11 @@
       <c r="O21">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P21" t="s">
+        <v>2185</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -8790,8 +8856,11 @@
       <c r="O22">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P22" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
@@ -8837,8 +8906,11 @@
       <c r="O23">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P23" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
@@ -8881,8 +8953,11 @@
       <c r="O24">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P24" t="s">
+        <v>2203</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>312</v>
       </c>
@@ -8925,8 +9000,11 @@
       <c r="O25">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P25" t="s">
+        <v>2204</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>23</v>
       </c>
@@ -8972,8 +9050,11 @@
       <c r="O26">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P26" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>24</v>
       </c>
@@ -9019,8 +9100,11 @@
       <c r="O27">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P27" t="s">
+        <v>2210</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>25</v>
       </c>
@@ -9066,8 +9150,11 @@
       <c r="O28">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P28" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>26</v>
       </c>
@@ -9113,8 +9200,11 @@
       <c r="O29">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P29" t="s">
+        <v>2214</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>27</v>
       </c>
@@ -9160,8 +9250,11 @@
       <c r="O30">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P30" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>28</v>
       </c>
@@ -9204,8 +9297,11 @@
       <c r="O31">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P31" t="s">
+        <v>2218</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>29</v>
       </c>
@@ -9251,8 +9347,11 @@
       <c r="O32">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P32" t="s">
+        <v>2223</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>30</v>
       </c>
@@ -9298,8 +9397,11 @@
       <c r="O33">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P33" t="s">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>31</v>
       </c>
@@ -9345,8 +9447,11 @@
       <c r="O34">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P34" t="s">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>32</v>
       </c>
@@ -9392,8 +9497,11 @@
       <c r="O35">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P35" t="s">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>33</v>
       </c>
@@ -9439,8 +9547,11 @@
       <c r="O36">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P36" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>34</v>
       </c>
@@ -9483,8 +9594,11 @@
       <c r="O37">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P37" t="s">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>35</v>
       </c>
@@ -9530,8 +9644,11 @@
       <c r="O38">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P38" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>319</v>
       </c>
@@ -9574,8 +9691,11 @@
       <c r="O39">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P39" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>320</v>
       </c>
@@ -9612,8 +9732,11 @@
       <c r="M40" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P40" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>36</v>
       </c>
@@ -9659,8 +9782,11 @@
       <c r="O41">
         <v>0.91</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P41" t="s">
+        <v>2109</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>37</v>
       </c>
@@ -9706,8 +9832,11 @@
       <c r="O42">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P42" t="s">
+        <v>2111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>38</v>
       </c>
@@ -9753,8 +9882,11 @@
       <c r="O43">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P43" t="s">
+        <v>2118</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>39</v>
       </c>
@@ -9800,8 +9932,11 @@
       <c r="O44">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P44" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>40</v>
       </c>
@@ -9844,8 +9979,11 @@
       <c r="O45">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P45" t="s">
+        <v>2134</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>41</v>
       </c>
@@ -9891,8 +10029,11 @@
       <c r="O46">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P46" t="s">
+        <v>2136</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>42</v>
       </c>
@@ -9938,8 +10079,11 @@
       <c r="O47">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P47" t="s">
+        <v>2140</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>43</v>
       </c>
@@ -9985,8 +10129,11 @@
       <c r="O48">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P48" t="s">
+        <v>2143</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>44</v>
       </c>
@@ -10029,8 +10176,11 @@
       <c r="O49">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P49" t="s">
+        <v>2144</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>307</v>
       </c>
@@ -10070,8 +10220,11 @@
       <c r="M50" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P50" t="s">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>45</v>
       </c>
@@ -10117,8 +10270,11 @@
       <c r="O51">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P51" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>46</v>
       </c>
@@ -10164,8 +10320,11 @@
       <c r="O52">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P52" t="s">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>47</v>
       </c>
@@ -10211,8 +10370,11 @@
       <c r="O53">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P53" t="s">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>48</v>
       </c>
@@ -10258,8 +10420,11 @@
       <c r="O54">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P54" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>49</v>
       </c>
@@ -10305,8 +10470,11 @@
       <c r="O55">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P55" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>50</v>
       </c>
@@ -10352,8 +10520,11 @@
       <c r="O56">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P56" t="s">
+        <v>2166</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>51</v>
       </c>
@@ -10399,8 +10570,11 @@
       <c r="O57">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P57" t="s">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>52</v>
       </c>
@@ -10446,8 +10620,11 @@
       <c r="O58">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P58" t="s">
+        <v>2174</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>53</v>
       </c>
@@ -10493,8 +10670,11 @@
       <c r="O59">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P59" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>54</v>
       </c>
@@ -10540,8 +10720,11 @@
       <c r="O60">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P60" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>55</v>
       </c>
@@ -10587,8 +10770,11 @@
       <c r="O61">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P61" t="s">
+        <v>2179</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>56</v>
       </c>
@@ -10634,8 +10820,11 @@
       <c r="O62">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P62" t="s">
+        <v>2181</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>57</v>
       </c>
@@ -10681,8 +10870,11 @@
       <c r="O63">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P63" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>58</v>
       </c>
@@ -10722,8 +10914,11 @@
       <c r="M64" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P64" t="s">
+        <v>2186</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>59</v>
       </c>
@@ -10766,8 +10961,11 @@
       <c r="O65">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P65" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>60</v>
       </c>
@@ -10813,8 +11011,11 @@
       <c r="O66">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P66" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>61</v>
       </c>
@@ -10860,8 +11061,11 @@
       <c r="O67">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P67" t="s">
+        <v>2195</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>62</v>
       </c>
@@ -10907,8 +11111,11 @@
       <c r="O68">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P68" t="s">
+        <v>2196</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>64</v>
       </c>
@@ -10954,8 +11161,11 @@
       <c r="O69">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P69" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>65</v>
       </c>
@@ -11001,8 +11211,11 @@
       <c r="O70">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P70" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>66</v>
       </c>
@@ -11048,8 +11261,11 @@
       <c r="O71">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P71" t="s">
+        <v>2216</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>67</v>
       </c>
@@ -11089,8 +11305,11 @@
       <c r="M72" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P72" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>68</v>
       </c>
@@ -11136,8 +11355,11 @@
       <c r="O73">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P73" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>69</v>
       </c>
@@ -11183,8 +11405,11 @@
       <c r="O74">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P74" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>70</v>
       </c>
@@ -11230,8 +11455,11 @@
       <c r="O75">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P75" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>289</v>
       </c>
@@ -11271,8 +11499,11 @@
       <c r="M76" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P76" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>71</v>
       </c>
@@ -11318,8 +11549,11 @@
       <c r="O77">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P77" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>72</v>
       </c>
@@ -11365,8 +11599,11 @@
       <c r="O78">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P78" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>313</v>
       </c>
@@ -11406,8 +11643,11 @@
       <c r="M79" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P79" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>73</v>
       </c>
@@ -11450,8 +11690,11 @@
       <c r="O80">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P80" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>75</v>
       </c>
@@ -11494,8 +11737,11 @@
       <c r="O81">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P81" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>76</v>
       </c>
@@ -11541,8 +11787,11 @@
       <c r="O82">
         <v>0.87</v>
       </c>
-    </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P82" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>77</v>
       </c>
@@ -11588,8 +11837,11 @@
       <c r="O83">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P83" t="s">
+        <v>2108</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>314</v>
       </c>
@@ -11632,8 +11884,11 @@
       <c r="N84">
         <v>0.35</v>
       </c>
-    </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P84" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>78</v>
       </c>
@@ -11679,8 +11934,11 @@
       <c r="O85">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P85" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>79</v>
       </c>
@@ -11726,8 +11984,11 @@
       <c r="O86">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P86" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>80</v>
       </c>
@@ -11773,8 +12034,11 @@
       <c r="O87">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P87" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>81</v>
       </c>
@@ -11820,8 +12084,11 @@
       <c r="O88">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P88" t="s">
+        <v>2203</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>82</v>
       </c>
@@ -11867,8 +12134,11 @@
       <c r="O89">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P89" t="s">
+        <v>2204</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>83</v>
       </c>
@@ -11914,8 +12184,11 @@
       <c r="O90">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P90" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>84</v>
       </c>
@@ -11961,8 +12234,11 @@
       <c r="O91">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P91" t="s">
+        <v>2210</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>85</v>
       </c>
@@ -12005,8 +12281,11 @@
       <c r="O92">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P92" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>86</v>
       </c>
@@ -12052,8 +12331,11 @@
       <c r="O93">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P93" t="s">
+        <v>2214</v>
+      </c>
+    </row>
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>87</v>
       </c>
@@ -12096,8 +12378,11 @@
       <c r="O94">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P94" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>88</v>
       </c>
@@ -12143,8 +12428,11 @@
       <c r="O95">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P95" t="s">
+        <v>2218</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>89</v>
       </c>
@@ -12190,8 +12478,11 @@
       <c r="O96">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P96" t="s">
+        <v>2223</v>
+      </c>
+    </row>
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>90</v>
       </c>
@@ -12237,8 +12528,11 @@
       <c r="O97">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P97" t="s">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>91</v>
       </c>
@@ -12284,8 +12578,11 @@
       <c r="O98">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P98" t="s">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>92</v>
       </c>
@@ -12328,8 +12625,11 @@
       <c r="O99">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P99" t="s">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>93</v>
       </c>
@@ -12375,8 +12675,11 @@
       <c r="O100">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P100" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>94</v>
       </c>
@@ -12422,8 +12725,11 @@
       <c r="O101">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P101" t="s">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>95</v>
       </c>
@@ -12463,8 +12769,11 @@
       <c r="M102" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P102" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>96</v>
       </c>
@@ -12510,8 +12819,11 @@
       <c r="O103">
         <v>0.81</v>
       </c>
-    </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P103" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>97</v>
       </c>
@@ -12557,8 +12869,11 @@
       <c r="O104">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P104" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>98</v>
       </c>
@@ -12604,8 +12919,11 @@
       <c r="O105">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P105" t="s">
+        <v>2109</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>99</v>
       </c>
@@ -12651,8 +12969,11 @@
       <c r="O106">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P106" t="s">
+        <v>2111</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>100</v>
       </c>
@@ -12698,8 +13019,11 @@
       <c r="O107">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P107" t="s">
+        <v>2118</v>
+      </c>
+    </row>
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>101</v>
       </c>
@@ -12745,8 +13069,11 @@
       <c r="O108">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P108" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>102</v>
       </c>
@@ -12792,8 +13119,11 @@
       <c r="O109">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P109" t="s">
+        <v>2134</v>
+      </c>
+    </row>
+    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>103</v>
       </c>
@@ -12839,8 +13169,11 @@
       <c r="O110">
         <v>0.89</v>
       </c>
-    </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P110" t="s">
+        <v>2136</v>
+      </c>
+    </row>
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>290</v>
       </c>
@@ -12880,8 +13213,11 @@
       <c r="M111" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P111" t="s">
+        <v>2140</v>
+      </c>
+    </row>
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>104</v>
       </c>
@@ -12927,8 +13263,11 @@
       <c r="O112">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P112" t="s">
+        <v>2143</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>105</v>
       </c>
@@ -12971,8 +13310,11 @@
       <c r="O113">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P113" t="s">
+        <v>2144</v>
+      </c>
+    </row>
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>106</v>
       </c>
@@ -13018,8 +13360,11 @@
       <c r="O114">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P114" t="s">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>107</v>
       </c>
@@ -13065,8 +13410,11 @@
       <c r="O115">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P115" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>108</v>
       </c>
@@ -13112,8 +13460,11 @@
       <c r="O116">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P116" t="s">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>109</v>
       </c>
@@ -13150,8 +13501,11 @@
       <c r="M117" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P117" t="s">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>110</v>
       </c>
@@ -13197,8 +13551,11 @@
       <c r="O118">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P118" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>111</v>
       </c>
@@ -13244,8 +13601,11 @@
       <c r="O119">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P119" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>112</v>
       </c>
@@ -13291,8 +13651,11 @@
       <c r="O120">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P120" t="s">
+        <v>2166</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>113</v>
       </c>
@@ -13338,8 +13701,11 @@
       <c r="O121">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P121" t="s">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>114</v>
       </c>
@@ -13385,8 +13751,11 @@
       <c r="O122">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P122" t="s">
+        <v>2174</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>115</v>
       </c>
@@ -13429,8 +13798,11 @@
       <c r="O123">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P123" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>116</v>
       </c>
@@ -13470,8 +13842,11 @@
       <c r="M124" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P124" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>300</v>
       </c>
@@ -13511,8 +13886,11 @@
       <c r="M125" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P125" t="s">
+        <v>2179</v>
+      </c>
+    </row>
+    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>117</v>
       </c>
@@ -13552,8 +13930,11 @@
       <c r="M126" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P126" t="s">
+        <v>2181</v>
+      </c>
+    </row>
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>118</v>
       </c>
@@ -13599,8 +13980,11 @@
       <c r="O127">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P127" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>119</v>
       </c>
@@ -13646,8 +14030,11 @@
       <c r="O128">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P128" t="s">
+        <v>2186</v>
+      </c>
+    </row>
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>120</v>
       </c>
@@ -13693,8 +14080,11 @@
       <c r="O129">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P129" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>121</v>
       </c>
@@ -13740,8 +14130,11 @@
       <c r="O130">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P130" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>122</v>
       </c>
@@ -13781,8 +14174,11 @@
       <c r="M131" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P131" t="s">
+        <v>2195</v>
+      </c>
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>123</v>
       </c>
@@ -13828,8 +14224,11 @@
       <c r="O132">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P132" t="s">
+        <v>2196</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>124</v>
       </c>
@@ -13875,8 +14274,11 @@
       <c r="O133">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P133" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>304</v>
       </c>
@@ -13916,8 +14318,11 @@
       <c r="M134" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P134" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>125</v>
       </c>
@@ -13963,8 +14368,11 @@
       <c r="O135">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P135" t="s">
+        <v>2216</v>
+      </c>
+    </row>
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>301</v>
       </c>
@@ -14004,8 +14412,11 @@
       <c r="M136" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P136" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>302</v>
       </c>
@@ -14045,8 +14456,11 @@
       <c r="M137" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P137" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>126</v>
       </c>
@@ -14092,8 +14506,11 @@
       <c r="O138">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P138" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>127</v>
       </c>
@@ -14136,8 +14553,11 @@
       <c r="O139">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P139" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>128</v>
       </c>
@@ -14183,8 +14603,11 @@
       <c r="O140">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P140" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>129</v>
       </c>
@@ -14230,8 +14653,11 @@
       <c r="O141">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P141" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>130</v>
       </c>
@@ -14277,8 +14703,11 @@
       <c r="O142">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P142" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>131</v>
       </c>
@@ -14324,8 +14753,11 @@
       <c r="O143">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P143" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>132</v>
       </c>
@@ -14368,8 +14800,11 @@
       <c r="O144">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P144" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>133</v>
       </c>
@@ -14415,8 +14850,11 @@
       <c r="O145">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P145" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>134</v>
       </c>
@@ -14462,8 +14900,11 @@
       <c r="O146">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P146" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>135</v>
       </c>
@@ -14506,8 +14947,11 @@
       <c r="O147">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P147" t="s">
+        <v>2108</v>
+      </c>
+    </row>
+    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>136</v>
       </c>
@@ -14553,8 +14997,11 @@
       <c r="O148">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P148" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>137</v>
       </c>
@@ -14600,8 +15047,11 @@
       <c r="O149">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P149" t="s">
+        <v>2212</v>
+      </c>
+    </row>
+    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>138</v>
       </c>
@@ -14647,8 +15097,11 @@
       <c r="O150">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P150" t="s">
+        <v>2109</v>
+      </c>
+    </row>
+    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>139</v>
       </c>
@@ -14694,8 +15147,11 @@
       <c r="O151">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P151" t="s">
+        <v>2111</v>
+      </c>
+    </row>
+    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>140</v>
       </c>
@@ -14741,8 +15197,11 @@
       <c r="O152">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P152" t="s">
+        <v>2118</v>
+      </c>
+    </row>
+    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>141</v>
       </c>
@@ -14785,8 +15244,11 @@
       <c r="O153">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P153" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>142</v>
       </c>
@@ -14832,8 +15294,11 @@
       <c r="O154">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P154" t="s">
+        <v>2134</v>
+      </c>
+    </row>
+    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>143</v>
       </c>
@@ -14879,8 +15344,11 @@
       <c r="O155">
         <v>0.67</v>
       </c>
-    </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P155" t="s">
+        <v>2136</v>
+      </c>
+    </row>
+    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>144</v>
       </c>
@@ -14926,8 +15394,11 @@
       <c r="O156">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P156" t="s">
+        <v>2140</v>
+      </c>
+    </row>
+    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>145</v>
       </c>
@@ -14970,8 +15441,11 @@
       <c r="O157">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P157" t="s">
+        <v>2143</v>
+      </c>
+    </row>
+    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>146</v>
       </c>
@@ -15017,8 +15491,11 @@
       <c r="O158">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P158" t="s">
+        <v>2144</v>
+      </c>
+    </row>
+    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>147</v>
       </c>
@@ -15064,8 +15541,11 @@
       <c r="O159">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P159" t="s">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>148</v>
       </c>
@@ -15111,8 +15591,11 @@
       <c r="O160">
         <v>0.91</v>
       </c>
-    </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P160" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="161" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>149</v>
       </c>
@@ -15158,8 +15641,11 @@
       <c r="O161">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P161" t="s">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="162" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>150</v>
       </c>
@@ -15205,8 +15691,11 @@
       <c r="O162">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P162" t="s">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="163" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>151</v>
       </c>
@@ -15252,8 +15741,11 @@
       <c r="O163">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P163" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="164" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>152</v>
       </c>
@@ -15299,8 +15791,11 @@
       <c r="O164">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P164" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="165" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>153</v>
       </c>
@@ -15346,8 +15841,11 @@
       <c r="O165">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P165" t="s">
+        <v>2166</v>
+      </c>
+    </row>
+    <row r="166" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>154</v>
       </c>
@@ -15393,8 +15891,11 @@
       <c r="O166">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P166" t="s">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="167" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>155</v>
       </c>
@@ -15440,8 +15941,11 @@
       <c r="O167">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P167" t="s">
+        <v>2174</v>
+      </c>
+    </row>
+    <row r="168" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>303</v>
       </c>
@@ -15484,8 +15988,11 @@
       <c r="N168">
         <v>0.65</v>
       </c>
-    </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P168" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="169" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>156</v>
       </c>
@@ -15531,8 +16038,11 @@
       <c r="O169">
         <v>0.83</v>
       </c>
-    </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P169" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>157</v>
       </c>
@@ -15578,8 +16088,11 @@
       <c r="O170">
         <v>0.83</v>
       </c>
-    </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P170" t="s">
+        <v>2179</v>
+      </c>
+    </row>
+    <row r="171" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>158</v>
       </c>
@@ -15622,8 +16135,11 @@
       <c r="O171">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P171" t="s">
+        <v>2181</v>
+      </c>
+    </row>
+    <row r="172" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>159</v>
       </c>
@@ -15669,8 +16185,11 @@
       <c r="O172">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P172" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="173" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>160</v>
       </c>
@@ -15716,8 +16235,11 @@
       <c r="O173">
         <v>0.84</v>
       </c>
-    </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P173" t="s">
+        <v>2186</v>
+      </c>
+    </row>
+    <row r="174" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>161</v>
       </c>
@@ -15763,8 +16285,11 @@
       <c r="O174">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P174" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="175" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>162</v>
       </c>
@@ -15810,8 +16335,11 @@
       <c r="O175">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P175" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="176" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>163</v>
       </c>
@@ -15857,8 +16385,11 @@
       <c r="O176">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P176" t="s">
+        <v>2195</v>
+      </c>
+    </row>
+    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>164</v>
       </c>
@@ -15904,8 +16435,11 @@
       <c r="O177">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P177" t="s">
+        <v>2196</v>
+      </c>
+    </row>
+    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>165</v>
       </c>
@@ -15951,8 +16485,11 @@
       <c r="O178">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P178" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>166</v>
       </c>
@@ -15998,8 +16535,11 @@
       <c r="O179">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P179" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>167</v>
       </c>
@@ -16045,8 +16585,11 @@
       <c r="O180">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P180" t="s">
+        <v>2216</v>
+      </c>
+    </row>
+    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>168</v>
       </c>
@@ -16092,8 +16635,11 @@
       <c r="O181">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P181" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>169</v>
       </c>
@@ -16139,8 +16685,11 @@
       <c r="O182">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P182" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>170</v>
       </c>
@@ -16183,8 +16732,11 @@
       <c r="O183">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P183" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>171</v>
       </c>
@@ -16230,8 +16782,11 @@
       <c r="O184">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P184" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>172</v>
       </c>
@@ -16277,8 +16832,11 @@
       <c r="O185">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P185" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>173</v>
       </c>
@@ -16324,8 +16882,11 @@
       <c r="O186">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P186" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>174</v>
       </c>
@@ -16368,8 +16929,11 @@
       <c r="O187">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P187" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>175</v>
       </c>
@@ -16415,8 +16979,11 @@
       <c r="O188">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P188" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>176</v>
       </c>
@@ -16462,8 +17029,11 @@
       <c r="O189">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P189" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>177</v>
       </c>
@@ -16509,8 +17079,11 @@
       <c r="O190">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P190" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>178</v>
       </c>
@@ -16556,8 +17129,11 @@
       <c r="O191">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P191" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>179</v>
       </c>
@@ -16603,8 +17179,11 @@
       <c r="O192">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P192" t="s">
+        <v>2108</v>
+      </c>
+    </row>
+    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>180</v>
       </c>
@@ -16650,8 +17229,11 @@
       <c r="O193">
         <v>0.81</v>
       </c>
-    </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P193" t="s">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>181</v>
       </c>
@@ -16697,8 +17279,11 @@
       <c r="O194">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P194" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>182</v>
       </c>
@@ -16744,8 +17329,11 @@
       <c r="O195">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P195" t="s">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>284</v>
       </c>
@@ -16785,8 +17373,11 @@
       <c r="M196" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P196" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>183</v>
       </c>
@@ -16832,8 +17423,11 @@
       <c r="O197">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P197" t="s">
+        <v>2228</v>
+      </c>
+    </row>
+    <row r="198" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>184</v>
       </c>
@@ -16879,8 +17473,11 @@
       <c r="O198">
         <v>0.81</v>
       </c>
-    </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P198" t="s">
+        <v>2124</v>
+      </c>
+    </row>
+    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>185</v>
       </c>
@@ -16926,8 +17523,11 @@
       <c r="O199">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P199" t="s">
+        <v>2261</v>
+      </c>
+    </row>
+    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>186</v>
       </c>
@@ -16973,8 +17573,11 @@
       <c r="O200">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P200" t="s">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>187</v>
       </c>
@@ -17020,8 +17623,11 @@
       <c r="O201">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P201" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>188</v>
       </c>
@@ -17064,8 +17670,11 @@
       <c r="O202">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P202" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="203" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>189</v>
       </c>
@@ -17111,8 +17720,11 @@
       <c r="O203">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P203" t="s">
+        <v>2233</v>
+      </c>
+    </row>
+    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>190</v>
       </c>
@@ -17158,8 +17770,11 @@
       <c r="O204">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P204" t="s">
+        <v>2191</v>
+      </c>
+    </row>
+    <row r="205" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>191</v>
       </c>
@@ -17205,8 +17820,11 @@
       <c r="O205">
         <v>0.87</v>
       </c>
-    </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P205" t="s">
+        <v>2186</v>
+      </c>
+    </row>
+    <row r="206" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>192</v>
       </c>
@@ -17252,8 +17870,11 @@
       <c r="O206">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P206" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="207" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>308</v>
       </c>
@@ -17293,8 +17914,11 @@
       <c r="M207" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P207" t="s">
+        <v>2166</v>
+      </c>
+    </row>
+    <row r="208" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>193</v>
       </c>
@@ -17340,8 +17964,11 @@
       <c r="O208">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P208" t="s">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="209" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>281</v>
       </c>
@@ -17381,8 +18008,11 @@
       <c r="M209" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P209" t="s">
+        <v>2172</v>
+      </c>
+    </row>
+    <row r="210" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>194</v>
       </c>
@@ -17428,8 +18058,11 @@
       <c r="O210">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P210" t="s">
+        <v>2135</v>
+      </c>
+    </row>
+    <row r="211" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>195</v>
       </c>
@@ -17475,8 +18108,11 @@
       <c r="O211">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P211" t="s">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="212" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>196</v>
       </c>
@@ -17522,8 +18158,11 @@
       <c r="O212">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P212" t="s">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="213" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>197</v>
       </c>
@@ -17569,8 +18208,11 @@
       <c r="O213">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P213" t="s">
+        <v>2151</v>
+      </c>
+    </row>
+    <row r="214" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>198</v>
       </c>
@@ -17616,8 +18258,11 @@
       <c r="O214">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P214" t="s">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="215" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>199</v>
       </c>
@@ -17663,8 +18308,11 @@
       <c r="O215">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P215" t="s">
+        <v>2174</v>
+      </c>
+    </row>
+    <row r="216" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>200</v>
       </c>
@@ -17710,8 +18358,11 @@
       <c r="O216">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P216" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="217" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>201</v>
       </c>
@@ -17757,8 +18408,11 @@
       <c r="O217">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P217" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="218" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>305</v>
       </c>
@@ -17798,8 +18452,11 @@
       <c r="M218" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P218" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="219" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>202</v>
       </c>
@@ -17845,8 +18502,11 @@
       <c r="O219">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="220" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P219" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="220" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>306</v>
       </c>
@@ -17886,8 +18546,11 @@
       <c r="M220" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="221" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P220" t="s">
+        <v>2179</v>
+      </c>
+    </row>
+    <row r="221" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>203</v>
       </c>
@@ -17933,8 +18596,11 @@
       <c r="O221">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="222" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P221" t="s">
+        <v>2138</v>
+      </c>
+    </row>
+    <row r="222" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>204</v>
       </c>
@@ -17980,8 +18646,11 @@
       <c r="O222">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="223" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P222" t="s">
+        <v>2181</v>
+      </c>
+    </row>
+    <row r="223" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>205</v>
       </c>
@@ -18027,8 +18696,11 @@
       <c r="O223">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="224" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P223" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="224" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>206</v>
       </c>
@@ -18074,8 +18746,11 @@
       <c r="O224">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="225" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P224" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="225" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>208</v>
       </c>
@@ -18121,8 +18796,11 @@
       <c r="O225">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="226" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P225" t="s">
+        <v>2173</v>
+      </c>
+    </row>
+    <row r="226" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>209</v>
       </c>
@@ -18165,8 +18843,11 @@
       <c r="O226">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="227" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P226" t="s">
+        <v>2141</v>
+      </c>
+    </row>
+    <row r="227" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>311</v>
       </c>
@@ -18209,8 +18890,11 @@
       <c r="O227">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="228" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P227" t="s">
+        <v>2186</v>
+      </c>
+    </row>
+    <row r="228" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>210</v>
       </c>
@@ -18256,8 +18940,11 @@
       <c r="O228">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="229" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P228" t="s">
+        <v>2151</v>
+      </c>
+    </row>
+    <row r="229" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>211</v>
       </c>
@@ -18303,8 +18990,11 @@
       <c r="O229">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="230" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P229" t="s">
+        <v>2185</v>
+      </c>
+    </row>
+    <row r="230" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>213</v>
       </c>
@@ -18347,8 +19037,11 @@
       <c r="O230">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="231" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P230" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="231" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>214</v>
       </c>
@@ -18394,8 +19087,11 @@
       <c r="O231">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="232" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P231" t="s">
+        <v>2194</v>
+      </c>
+    </row>
+    <row r="232" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>215</v>
       </c>
@@ -18441,8 +19137,11 @@
       <c r="O232">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="233" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P232" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="233" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>216</v>
       </c>
@@ -18488,8 +19187,11 @@
       <c r="O233">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="234" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P233" t="s">
+        <v>2139</v>
+      </c>
+    </row>
+    <row r="234" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>287</v>
       </c>
@@ -18529,8 +19231,11 @@
       <c r="M234" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="235" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P234" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="235" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>217</v>
       </c>
@@ -18576,8 +19281,11 @@
       <c r="O235">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="236" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P235" t="s">
+        <v>2146</v>
+      </c>
+    </row>
+    <row r="236" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>218</v>
       </c>
@@ -18623,8 +19331,11 @@
       <c r="O236">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="237" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P236" t="s">
+        <v>2195</v>
+      </c>
+    </row>
+    <row r="237" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>219</v>
       </c>
@@ -18670,8 +19381,11 @@
       <c r="O237">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="238" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P237" t="s">
+        <v>2196</v>
+      </c>
+    </row>
+    <row r="238" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>220</v>
       </c>
@@ -18714,8 +19428,11 @@
       <c r="O238">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="239" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P238" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="239" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>221</v>
       </c>
@@ -18761,8 +19478,11 @@
       <c r="O239">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="240" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P239" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="240" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>222</v>
       </c>
@@ -18805,8 +19525,11 @@
       <c r="O240">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="241" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P240" t="s">
+        <v>2207</v>
+      </c>
+    </row>
+    <row r="241" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>223</v>
       </c>
@@ -18852,8 +19575,11 @@
       <c r="O241">
         <v>0.81</v>
       </c>
-    </row>
-    <row r="242" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P241" t="s">
+        <v>2118</v>
+      </c>
+    </row>
+    <row r="242" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>224</v>
       </c>
@@ -18899,8 +19625,11 @@
       <c r="O242">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="243" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P242" t="s">
+        <v>2156</v>
+      </c>
+    </row>
+    <row r="243" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>225</v>
       </c>
@@ -18946,8 +19675,11 @@
       <c r="O243">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="244" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P243" t="s">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="244" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>286</v>
       </c>
@@ -18987,8 +19719,11 @@
       <c r="M244" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="245" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P244" t="s">
+        <v>2174</v>
+      </c>
+    </row>
+    <row r="245" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>227</v>
       </c>
@@ -19028,8 +19763,11 @@
       <c r="M245" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="246" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P245" t="s">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="246" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>228</v>
       </c>
@@ -19069,8 +19807,11 @@
       <c r="M246" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="247" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P246" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="247" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>229</v>
       </c>
@@ -19116,8 +19857,11 @@
       <c r="O247">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="248" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P247" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="248" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>231</v>
       </c>
@@ -19163,8 +19907,11 @@
       <c r="O248">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="249" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P248" t="s">
+        <v>2214</v>
+      </c>
+    </row>
+    <row r="249" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>232</v>
       </c>
@@ -19210,8 +19957,11 @@
       <c r="O249">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="250" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P249" t="s">
+        <v>2140</v>
+      </c>
+    </row>
+    <row r="250" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>233</v>
       </c>
@@ -19254,8 +20004,11 @@
       <c r="O250">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="251" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P250" t="s">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="251" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>230</v>
       </c>
@@ -19301,8 +20054,11 @@
       <c r="O251">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="252" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P251" t="s">
+        <v>2252</v>
+      </c>
+    </row>
+    <row r="252" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>234</v>
       </c>
@@ -19348,8 +20104,11 @@
       <c r="O252">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="253" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P252" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="253" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>235</v>
       </c>
@@ -19395,8 +20154,11 @@
       <c r="O253">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="254" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P253" t="s">
+        <v>2196</v>
+      </c>
+    </row>
+    <row r="254" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>236</v>
       </c>
@@ -19433,8 +20195,11 @@
       <c r="M254" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="255" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P254" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="255" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>237</v>
       </c>
@@ -19480,8 +20245,11 @@
       <c r="O255">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="256" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P255" t="s">
+        <v>2132</v>
+      </c>
+    </row>
+    <row r="256" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>238</v>
       </c>
@@ -19527,8 +20295,11 @@
       <c r="O256">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="257" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P256" t="s">
+        <v>2126</v>
+      </c>
+    </row>
+    <row r="257" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>239</v>
       </c>
@@ -19574,8 +20345,11 @@
       <c r="O257">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="258" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P257" t="s">
+        <v>2216</v>
+      </c>
+    </row>
+    <row r="258" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>240</v>
       </c>
@@ -19621,8 +20395,11 @@
       <c r="O258">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="259" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P258" t="s">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="259" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>241</v>
       </c>
@@ -19668,8 +20445,11 @@
       <c r="O259">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="260" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P259" t="s">
+        <v>2224</v>
+      </c>
+    </row>
+    <row r="260" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>242</v>
       </c>
@@ -19715,8 +20495,11 @@
       <c r="O260">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="261" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P260" t="s">
+        <v>2128</v>
+      </c>
+    </row>
+    <row r="261" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>243</v>
       </c>
@@ -19759,8 +20542,11 @@
       <c r="O261">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="262" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P261" t="s">
+        <v>2221</v>
+      </c>
+    </row>
+    <row r="262" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>244</v>
       </c>
@@ -19806,8 +20592,11 @@
       <c r="O262">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="263" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P262" t="s">
+        <v>2256</v>
+      </c>
+    </row>
+    <row r="263" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>283</v>
       </c>
@@ -19847,8 +20636,11 @@
       <c r="M263" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="264" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P263" t="s">
+        <v>2229</v>
+      </c>
+    </row>
+    <row r="264" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>246</v>
       </c>
@@ -19894,8 +20686,11 @@
       <c r="O264">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="265" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P264" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="265" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>247</v>
       </c>
@@ -19938,8 +20733,11 @@
       <c r="O265">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="266" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P265" t="s">
+        <v>2142</v>
+      </c>
+    </row>
+    <row r="266" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>248</v>
       </c>
@@ -19985,8 +20783,11 @@
       <c r="O266">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="267" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P266" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="267" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>249</v>
       </c>
@@ -20032,8 +20833,11 @@
       <c r="O267">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="268" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P267" t="s">
+        <v>2230</v>
+      </c>
+    </row>
+    <row r="268" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>250</v>
       </c>
@@ -20079,8 +20883,11 @@
       <c r="O268">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="269" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P268" t="s">
+        <v>2190</v>
+      </c>
+    </row>
+    <row r="269" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>252</v>
       </c>
@@ -20126,8 +20933,11 @@
       <c r="O269">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="270" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P269" t="s">
+        <v>2113</v>
+      </c>
+    </row>
+    <row r="270" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>253</v>
       </c>
@@ -20173,8 +20983,11 @@
       <c r="O270">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="271" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P270" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="271" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>254</v>
       </c>
@@ -20214,8 +21027,11 @@
       <c r="M271" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="272" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P271" t="s">
+        <v>2128</v>
+      </c>
+    </row>
+    <row r="272" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>255</v>
       </c>
@@ -20258,8 +21074,11 @@
       <c r="O272">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="273" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P272" t="s">
+        <v>2204</v>
+      </c>
+    </row>
+    <row r="273" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>256</v>
       </c>
@@ -20305,8 +21124,11 @@
       <c r="O273">
         <v>0.91</v>
       </c>
-    </row>
-    <row r="274" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P273" t="s">
+        <v>2123</v>
+      </c>
+    </row>
+    <row r="274" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>257</v>
       </c>
@@ -20352,8 +21174,11 @@
       <c r="O274">
         <v>0.91</v>
       </c>
-    </row>
-    <row r="275" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P274" t="s">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="275" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>310</v>
       </c>
@@ -20393,8 +21218,11 @@
       <c r="M275" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="276" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P275" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="276" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>258</v>
       </c>
@@ -20437,8 +21265,11 @@
       <c r="O276">
         <v>0.91</v>
       </c>
-    </row>
-    <row r="277" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P276" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="277" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>285</v>
       </c>
@@ -20478,8 +21309,11 @@
       <c r="M277" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="278" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P277" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="278" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>226</v>
       </c>
@@ -20525,8 +21359,11 @@
       <c r="O278">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="279" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P278" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="279" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>259</v>
       </c>
@@ -20572,8 +21409,11 @@
       <c r="O279">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="280" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P279" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="280" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>316</v>
       </c>
@@ -20613,8 +21453,11 @@
       <c r="M280" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="281" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P280" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="281" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>260</v>
       </c>
@@ -20660,8 +21503,11 @@
       <c r="O281">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="282" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P281" t="s">
+        <v>2114</v>
+      </c>
+    </row>
+    <row r="282" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>315</v>
       </c>
@@ -20701,8 +21547,11 @@
       <c r="M282" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="283" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P282" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="283" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>261</v>
       </c>
@@ -20748,8 +21597,11 @@
       <c r="O283">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="284" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P283" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="284" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>262</v>
       </c>
@@ -20795,8 +21647,11 @@
       <c r="O284">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="285" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P284" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="285" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>263</v>
       </c>
@@ -20842,8 +21697,11 @@
       <c r="O285">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="286" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P285" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="286" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>317</v>
       </c>
@@ -20883,8 +21741,11 @@
       <c r="M286" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="287" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P286" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="287" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>264</v>
       </c>
@@ -20930,8 +21791,11 @@
       <c r="O287">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="288" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P287" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="288" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>265</v>
       </c>
@@ -20977,8 +21841,11 @@
       <c r="O288">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="289" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P288" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="289" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>266</v>
       </c>
@@ -21024,8 +21891,11 @@
       <c r="O289">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="290" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P289" t="s">
+        <v>2125</v>
+      </c>
+    </row>
+    <row r="290" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>267</v>
       </c>
@@ -21071,8 +21941,11 @@
       <c r="O290">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="291" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P290" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="291" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>269</v>
       </c>
@@ -21115,8 +21988,11 @@
       <c r="O291">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="292" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P291" t="s">
+        <v>2201</v>
+      </c>
+    </row>
+    <row r="292" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>270</v>
       </c>
@@ -21162,8 +22038,11 @@
       <c r="O292">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="293" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P292" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="293" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>271</v>
       </c>
@@ -21209,8 +22088,11 @@
       <c r="O293">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="294" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P293" t="s">
+        <v>2144</v>
+      </c>
+    </row>
+    <row r="294" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>272</v>
       </c>
@@ -21256,8 +22138,11 @@
       <c r="O294">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="295" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P294" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="295" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>212</v>
       </c>
@@ -21297,8 +22182,11 @@
       <c r="M295" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="296" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P295" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="296" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>274</v>
       </c>
@@ -21344,8 +22232,11 @@
       <c r="O296">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="297" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P296" t="s">
+        <v>2108</v>
+      </c>
+    </row>
+    <row r="297" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>275</v>
       </c>
@@ -21391,8 +22282,11 @@
       <c r="O297">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="298" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P297" t="s">
+        <v>2164</v>
+      </c>
+    </row>
+    <row r="298" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>276</v>
       </c>
@@ -21438,8 +22332,11 @@
       <c r="O298">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="299" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P298" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="299" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>277</v>
       </c>
@@ -21485,8 +22382,11 @@
       <c r="O299">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="300" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P299" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="300" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>278</v>
       </c>
@@ -21529,8 +22429,11 @@
       <c r="O300">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="301" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P300" t="s">
+        <v>2168</v>
+      </c>
+    </row>
+    <row r="301" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>309</v>
       </c>
@@ -21569,6 +22472,9 @@
       </c>
       <c r="M301" t="s">
         <v>36</v>
+      </c>
+      <c r="P301" t="s">
+        <v>2268</v>
       </c>
     </row>
   </sheetData>
@@ -55405,7 +56311,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:BM301"/>
+  <dimension ref="A1:BM300"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
@@ -96966,11 +97872,6 @@
         <v>2168</v>
       </c>
     </row>
-    <row r="301" spans="1:65" x14ac:dyDescent="0.25">
-      <c r="BM301" t="s">
-        <v>2223</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="AC1:AC300" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:BK300">

</xml_diff>

<commit_message>
Uh I don't know
</commit_message>
<xml_diff>
--- a/NWspecies060222.xlsx
+++ b/NWspecies060222.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0f4fad9919cbe5b/Neighbourwoods/NWAnalytics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="8_{DD247510-64D4-4C56-90AC-C75474531547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D35ADC4-AD9E-4400-91C2-0CA214A1A8D0}"/>
+  <xr:revisionPtr revIDLastSave="121" documentId="8_{DD247510-64D4-4C56-90AC-C75474531547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39C1BF07-830D-4D89-AAE0-FCD9D2CA1881}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="species" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'all data'!$AC$1:$AC$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">colors!$A$1:$A$335</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">species!$L$1:$L$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">species!$B$1:$B$301</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
various additions to NWAnalytics3 and some edits to species names in spp table
</commit_message>
<xml_diff>
--- a/NWspecies060222.xlsx
+++ b/NWspecies060222.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0f4fad9919cbe5b/Neighbourwoods/NWAnalytics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="8_{DD247510-64D4-4C56-90AC-C75474531547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C438AE63-C5C7-486A-9C10-4BCDB06FEA7A}"/>
+  <xr:revisionPtr revIDLastSave="130" documentId="8_{DD247510-64D4-4C56-90AC-C75474531547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B4B925E-0931-4367-B949-35B724ECC164}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'all data'!$AC$1:$AC$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">colors!$A$1:$A$335</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">species!$B$1:$B$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">species!$L$1:$L$301</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -7779,12 +7779,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Sheet1"/>
+  <sheetPr codeName="Sheet1" filterMode="1"/>
   <dimension ref="A1:P301"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.140625" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" customWidth="1"/>
     <col min="5" max="5" width="27" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="28.5703125" customWidth="1"/>
@@ -7846,7 +7847,7 @@
         <v>2107</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7896,7 +7897,7 @@
         <v>2108</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7946,7 +7947,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7993,7 +7994,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -8043,7 +8044,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>318</v>
       </c>
@@ -8087,7 +8088,7 @@
         <v>2121</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -8131,7 +8132,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -8181,7 +8182,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -8225,7 +8226,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>282</v>
       </c>
@@ -8269,7 +8270,7 @@
         <v>2146</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -8319,7 +8320,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -8369,7 +8370,7 @@
         <v>2152</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -8419,7 +8420,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -8469,7 +8470,7 @@
         <v>2156</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -8519,7 +8520,7 @@
         <v>2161</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -8566,7 +8567,7 @@
         <v>2163</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -8616,7 +8617,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -8666,7 +8667,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -8716,7 +8717,7 @@
         <v>2182</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -8766,7 +8767,7 @@
         <v>2184</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -8816,7 +8817,7 @@
         <v>2185</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -8866,7 +8867,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
@@ -8916,7 +8917,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
@@ -8963,7 +8964,7 @@
         <v>2203</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>312</v>
       </c>
@@ -9010,7 +9011,7 @@
         <v>2204</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>23</v>
       </c>
@@ -9060,7 +9061,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>24</v>
       </c>
@@ -9110,7 +9111,7 @@
         <v>2210</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>25</v>
       </c>
@@ -9160,7 +9161,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>26</v>
       </c>
@@ -9210,7 +9211,7 @@
         <v>2214</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>27</v>
       </c>
@@ -9260,7 +9261,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>28</v>
       </c>
@@ -9307,7 +9308,7 @@
         <v>2218</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>29</v>
       </c>
@@ -9357,7 +9358,7 @@
         <v>2223</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>30</v>
       </c>
@@ -9407,7 +9408,7 @@
         <v>2225</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>31</v>
       </c>
@@ -9457,7 +9458,7 @@
         <v>2226</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>32</v>
       </c>
@@ -9507,7 +9508,7 @@
         <v>2240</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>33</v>
       </c>
@@ -9557,7 +9558,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>34</v>
       </c>
@@ -9604,7 +9605,7 @@
         <v>2243</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>35</v>
       </c>
@@ -9654,7 +9655,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>319</v>
       </c>
@@ -9701,7 +9702,7 @@
         <v>2246</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>320</v>
       </c>
@@ -9742,7 +9743,7 @@
         <v>2249</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>36</v>
       </c>
@@ -9792,7 +9793,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>37</v>
       </c>
@@ -9842,7 +9843,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>38</v>
       </c>
@@ -9892,7 +9893,7 @@
         <v>2118</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>39</v>
       </c>
@@ -9942,7 +9943,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>40</v>
       </c>
@@ -9989,7 +9990,7 @@
         <v>2134</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>41</v>
       </c>
@@ -10039,7 +10040,7 @@
         <v>2136</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>42</v>
       </c>
@@ -10089,7 +10090,7 @@
         <v>2140</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>43</v>
       </c>
@@ -10139,7 +10140,7 @@
         <v>2143</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>44</v>
       </c>
@@ -10186,7 +10187,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>307</v>
       </c>
@@ -10230,7 +10231,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>45</v>
       </c>
@@ -10280,7 +10281,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>46</v>
       </c>
@@ -10330,7 +10331,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>47</v>
       </c>
@@ -10380,7 +10381,7 @@
         <v>2159</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>48</v>
       </c>
@@ -10430,7 +10431,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>49</v>
       </c>
@@ -10480,7 +10481,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>50</v>
       </c>
@@ -10530,7 +10531,7 @@
         <v>2166</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>51</v>
       </c>
@@ -10580,7 +10581,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>52</v>
       </c>
@@ -10630,7 +10631,7 @@
         <v>2174</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>53</v>
       </c>
@@ -10680,7 +10681,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>54</v>
       </c>
@@ -10730,7 +10731,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>55</v>
       </c>
@@ -10780,7 +10781,7 @@
         <v>2179</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>56</v>
       </c>
@@ -10830,7 +10831,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>57</v>
       </c>
@@ -10880,7 +10881,7 @@
         <v>2182</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>58</v>
       </c>
@@ -10924,7 +10925,7 @@
         <v>2186</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>59</v>
       </c>
@@ -10971,7 +10972,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>60</v>
       </c>
@@ -11021,7 +11022,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>61</v>
       </c>
@@ -11071,7 +11072,7 @@
         <v>2195</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>62</v>
       </c>
@@ -11121,7 +11122,7 @@
         <v>2196</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>64</v>
       </c>
@@ -11171,7 +11172,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>65</v>
       </c>
@@ -11221,7 +11222,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>66</v>
       </c>
@@ -11315,7 +11316,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>68</v>
       </c>
@@ -11365,7 +11366,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>69</v>
       </c>
@@ -11415,7 +11416,7 @@
         <v>2239</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>70</v>
       </c>
@@ -11465,7 +11466,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>289</v>
       </c>
@@ -11509,7 +11510,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>71</v>
       </c>
@@ -11559,7 +11560,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>72</v>
       </c>
@@ -11609,7 +11610,7 @@
         <v>2245</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>313</v>
       </c>
@@ -11653,7 +11654,7 @@
         <v>2246</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>73</v>
       </c>
@@ -11700,7 +11701,7 @@
         <v>2247</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>75</v>
       </c>
@@ -11747,7 +11748,7 @@
         <v>2249</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>76</v>
       </c>
@@ -11797,7 +11798,7 @@
         <v>2251</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>77</v>
       </c>
@@ -11847,7 +11848,7 @@
         <v>2108</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>314</v>
       </c>
@@ -11894,7 +11895,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>78</v>
       </c>
@@ -11944,7 +11945,7 @@
         <v>2231</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>79</v>
       </c>
@@ -11994,7 +11995,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>80</v>
       </c>
@@ -12044,7 +12045,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>81</v>
       </c>
@@ -12094,7 +12095,7 @@
         <v>2203</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>82</v>
       </c>
@@ -12144,7 +12145,7 @@
         <v>2204</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>83</v>
       </c>
@@ -12194,7 +12195,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>84</v>
       </c>
@@ -12244,7 +12245,7 @@
         <v>2210</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>85</v>
       </c>
@@ -12291,7 +12292,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>86</v>
       </c>
@@ -12341,7 +12342,7 @@
         <v>2214</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>87</v>
       </c>
@@ -12388,7 +12389,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>88</v>
       </c>
@@ -12438,7 +12439,7 @@
         <v>2218</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>89</v>
       </c>
@@ -12488,7 +12489,7 @@
         <v>2223</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>90</v>
       </c>
@@ -12538,7 +12539,7 @@
         <v>2225</v>
       </c>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>91</v>
       </c>
@@ -12588,7 +12589,7 @@
         <v>2226</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>92</v>
       </c>
@@ -12635,7 +12636,7 @@
         <v>2240</v>
       </c>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>93</v>
       </c>
@@ -12685,7 +12686,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>94</v>
       </c>
@@ -12779,7 +12780,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>96</v>
       </c>
@@ -12829,7 +12830,7 @@
         <v>2246</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>97</v>
       </c>
@@ -12879,7 +12880,7 @@
         <v>2249</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>98</v>
       </c>
@@ -12929,7 +12930,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>99</v>
       </c>
@@ -12979,7 +12980,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>100</v>
       </c>
@@ -13029,7 +13030,7 @@
         <v>2118</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>101</v>
       </c>
@@ -13079,7 +13080,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>102</v>
       </c>
@@ -13129,7 +13130,7 @@
         <v>2134</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>103</v>
       </c>
@@ -13179,7 +13180,7 @@
         <v>2136</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>290</v>
       </c>
@@ -13223,7 +13224,7 @@
         <v>2140</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>104</v>
       </c>
@@ -13273,7 +13274,7 @@
         <v>2143</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>105</v>
       </c>
@@ -13320,7 +13321,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>106</v>
       </c>
@@ -13370,7 +13371,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>107</v>
       </c>
@@ -13420,7 +13421,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>108</v>
       </c>
@@ -13511,7 +13512,7 @@
         <v>2159</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>110</v>
       </c>
@@ -13561,7 +13562,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>111</v>
       </c>
@@ -13611,7 +13612,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>112</v>
       </c>
@@ -13661,7 +13662,7 @@
         <v>2166</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>113</v>
       </c>
@@ -13711,7 +13712,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>114</v>
       </c>
@@ -13761,7 +13762,7 @@
         <v>2174</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>115</v>
       </c>
@@ -13808,7 +13809,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>116</v>
       </c>
@@ -13852,7 +13853,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>300</v>
       </c>
@@ -13896,7 +13897,7 @@
         <v>2179</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>117</v>
       </c>
@@ -13940,7 +13941,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>118</v>
       </c>
@@ -13990,7 +13991,7 @@
         <v>2182</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>119</v>
       </c>
@@ -14040,7 +14041,7 @@
         <v>2186</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>120</v>
       </c>
@@ -14090,7 +14091,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>121</v>
       </c>
@@ -14140,7 +14141,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>122</v>
       </c>
@@ -14184,7 +14185,7 @@
         <v>2195</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>123</v>
       </c>
@@ -14234,7 +14235,7 @@
         <v>2196</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>124</v>
       </c>
@@ -14284,7 +14285,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>304</v>
       </c>
@@ -14328,7 +14329,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>125</v>
       </c>
@@ -14378,7 +14379,7 @@
         <v>2216</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>301</v>
       </c>
@@ -14422,7 +14423,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>302</v>
       </c>
@@ -14466,7 +14467,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>126</v>
       </c>
@@ -14516,7 +14517,7 @@
         <v>2239</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>127</v>
       </c>
@@ -14563,7 +14564,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>128</v>
       </c>
@@ -14613,7 +14614,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>129</v>
       </c>
@@ -14663,7 +14664,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>130</v>
       </c>
@@ -14713,7 +14714,7 @@
         <v>2245</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>131</v>
       </c>
@@ -14763,7 +14764,7 @@
         <v>2246</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>132</v>
       </c>
@@ -14810,7 +14811,7 @@
         <v>2247</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>133</v>
       </c>
@@ -14860,7 +14861,7 @@
         <v>2249</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>134</v>
       </c>
@@ -14910,7 +14911,7 @@
         <v>2251</v>
       </c>
     </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>135</v>
       </c>
@@ -14957,7 +14958,7 @@
         <v>2108</v>
       </c>
     </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>136</v>
       </c>
@@ -15007,7 +15008,7 @@
         <v>2205</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>137</v>
       </c>
@@ -15057,7 +15058,7 @@
         <v>2212</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>138</v>
       </c>
@@ -15107,7 +15108,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>139</v>
       </c>
@@ -15157,7 +15158,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>140</v>
       </c>
@@ -15207,7 +15208,7 @@
         <v>2118</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>141</v>
       </c>
@@ -15254,7 +15255,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>142</v>
       </c>
@@ -15304,7 +15305,7 @@
         <v>2134</v>
       </c>
     </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>143</v>
       </c>
@@ -15354,7 +15355,7 @@
         <v>2136</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>144</v>
       </c>
@@ -15404,7 +15405,7 @@
         <v>2140</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>145</v>
       </c>
@@ -15451,7 +15452,7 @@
         <v>2143</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>146</v>
       </c>
@@ -15501,7 +15502,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>147</v>
       </c>
@@ -15551,7 +15552,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>148</v>
       </c>
@@ -15601,7 +15602,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>149</v>
       </c>
@@ -15651,7 +15652,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="162" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>150</v>
       </c>
@@ -15701,7 +15702,7 @@
         <v>2159</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>151</v>
       </c>
@@ -15751,7 +15752,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>152</v>
       </c>
@@ -15801,7 +15802,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>153</v>
       </c>
@@ -15851,7 +15852,7 @@
         <v>2166</v>
       </c>
     </row>
-    <row r="166" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>154</v>
       </c>
@@ -15901,7 +15902,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>155</v>
       </c>
@@ -15951,7 +15952,7 @@
         <v>2174</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>303</v>
       </c>
@@ -15998,7 +15999,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>156</v>
       </c>
@@ -16048,7 +16049,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>157</v>
       </c>
@@ -16098,7 +16099,7 @@
         <v>2179</v>
       </c>
     </row>
-    <row r="171" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>158</v>
       </c>
@@ -16145,7 +16146,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>159</v>
       </c>
@@ -16195,7 +16196,7 @@
         <v>2182</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>160</v>
       </c>
@@ -16245,7 +16246,7 @@
         <v>2186</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>161</v>
       </c>
@@ -16295,7 +16296,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>162</v>
       </c>
@@ -16345,7 +16346,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>163</v>
       </c>
@@ -16395,7 +16396,7 @@
         <v>2195</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>164</v>
       </c>
@@ -16445,7 +16446,7 @@
         <v>2196</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>165</v>
       </c>
@@ -16495,7 +16496,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>166</v>
       </c>
@@ -16545,7 +16546,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>167</v>
       </c>
@@ -16595,7 +16596,7 @@
         <v>2216</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>168</v>
       </c>
@@ -16645,7 +16646,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>169</v>
       </c>
@@ -16695,7 +16696,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>170</v>
       </c>
@@ -16742,7 +16743,7 @@
         <v>2239</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>171</v>
       </c>
@@ -16792,7 +16793,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>172</v>
       </c>
@@ -16842,7 +16843,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>173</v>
       </c>
@@ -16892,7 +16893,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>174</v>
       </c>
@@ -16939,7 +16940,7 @@
         <v>2245</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>175</v>
       </c>
@@ -16989,7 +16990,7 @@
         <v>2246</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>176</v>
       </c>
@@ -17039,7 +17040,7 @@
         <v>2247</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>177</v>
       </c>
@@ -17089,7 +17090,7 @@
         <v>2249</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>178</v>
       </c>
@@ -17139,7 +17140,7 @@
         <v>2251</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>179</v>
       </c>
@@ -17189,7 +17190,7 @@
         <v>2108</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>180</v>
       </c>
@@ -17239,7 +17240,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>181</v>
       </c>
@@ -17289,7 +17290,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>182</v>
       </c>
@@ -17339,7 +17340,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>284</v>
       </c>
@@ -17383,7 +17384,7 @@
         <v>2169</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>183</v>
       </c>
@@ -17433,7 +17434,7 @@
         <v>2228</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>184</v>
       </c>
@@ -17483,7 +17484,7 @@
         <v>2124</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>185</v>
       </c>
@@ -17533,7 +17534,7 @@
         <v>2261</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>186</v>
       </c>
@@ -17583,7 +17584,7 @@
         <v>2159</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>187</v>
       </c>
@@ -17633,7 +17634,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>188</v>
       </c>
@@ -17680,7 +17681,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>189</v>
       </c>
@@ -17730,7 +17731,7 @@
         <v>2233</v>
       </c>
     </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>190</v>
       </c>
@@ -17780,7 +17781,7 @@
         <v>2191</v>
       </c>
     </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>191</v>
       </c>
@@ -17830,7 +17831,7 @@
         <v>2186</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>192</v>
       </c>
@@ -17880,7 +17881,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>308</v>
       </c>
@@ -17924,7 +17925,7 @@
         <v>2166</v>
       </c>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>193</v>
       </c>
@@ -17974,7 +17975,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>281</v>
       </c>
@@ -18018,7 +18019,7 @@
         <v>2172</v>
       </c>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>194</v>
       </c>
@@ -18068,7 +18069,7 @@
         <v>2135</v>
       </c>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>195</v>
       </c>
@@ -18118,7 +18119,7 @@
         <v>2150</v>
       </c>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>196</v>
       </c>
@@ -18168,7 +18169,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>197</v>
       </c>
@@ -18218,7 +18219,7 @@
         <v>2151</v>
       </c>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>198</v>
       </c>
@@ -18268,7 +18269,7 @@
         <v>2226</v>
       </c>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>199</v>
       </c>
@@ -18318,7 +18319,7 @@
         <v>2174</v>
       </c>
     </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>200</v>
       </c>
@@ -18368,7 +18369,7 @@
         <v>2130</v>
       </c>
     </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>201</v>
       </c>
@@ -18418,7 +18419,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>305</v>
       </c>
@@ -18462,7 +18463,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>202</v>
       </c>
@@ -18512,7 +18513,7 @@
         <v>2251</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>306</v>
       </c>
@@ -18556,7 +18557,7 @@
         <v>2179</v>
       </c>
     </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>203</v>
       </c>
@@ -18606,7 +18607,7 @@
         <v>2138</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>204</v>
       </c>
@@ -18656,7 +18657,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>205</v>
       </c>
@@ -18706,7 +18707,7 @@
         <v>2182</v>
       </c>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>206</v>
       </c>
@@ -18756,7 +18757,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>208</v>
       </c>
@@ -18806,7 +18807,7 @@
         <v>2173</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>209</v>
       </c>
@@ -18853,7 +18854,7 @@
         <v>2141</v>
       </c>
     </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>311</v>
       </c>
@@ -18900,7 +18901,7 @@
         <v>2186</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>210</v>
       </c>
@@ -18950,7 +18951,7 @@
         <v>2151</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>211</v>
       </c>
@@ -19000,7 +19001,7 @@
         <v>2185</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>213</v>
       </c>
@@ -19047,7 +19048,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>214</v>
       </c>
@@ -19097,7 +19098,7 @@
         <v>2194</v>
       </c>
     </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>215</v>
       </c>
@@ -19147,7 +19148,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>216</v>
       </c>
@@ -19197,7 +19198,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>287</v>
       </c>
@@ -19241,7 +19242,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>217</v>
       </c>
@@ -19291,7 +19292,7 @@
         <v>2146</v>
       </c>
     </row>
-    <row r="236" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>218</v>
       </c>
@@ -19341,7 +19342,7 @@
         <v>2195</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>219</v>
       </c>
@@ -19391,7 +19392,7 @@
         <v>2196</v>
       </c>
     </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>220</v>
       </c>
@@ -19438,7 +19439,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="239" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>221</v>
       </c>
@@ -19488,7 +19489,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="240" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>222</v>
       </c>
@@ -19535,7 +19536,7 @@
         <v>2207</v>
       </c>
     </row>
-    <row r="241" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>223</v>
       </c>
@@ -19585,7 +19586,7 @@
         <v>2118</v>
       </c>
     </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>224</v>
       </c>
@@ -19635,7 +19636,7 @@
         <v>2156</v>
       </c>
     </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>225</v>
       </c>
@@ -19685,7 +19686,7 @@
         <v>2243</v>
       </c>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>286</v>
       </c>
@@ -19729,7 +19730,7 @@
         <v>2174</v>
       </c>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>227</v>
       </c>
@@ -19773,7 +19774,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>228</v>
       </c>
@@ -19817,7 +19818,7 @@
         <v>2247</v>
       </c>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>229</v>
       </c>
@@ -19867,7 +19868,7 @@
         <v>2127</v>
       </c>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>231</v>
       </c>
@@ -19917,7 +19918,7 @@
         <v>2214</v>
       </c>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>232</v>
       </c>
@@ -19967,7 +19968,7 @@
         <v>2140</v>
       </c>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>233</v>
       </c>
@@ -20014,7 +20015,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>230</v>
       </c>
@@ -20064,7 +20065,7 @@
         <v>2252</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>234</v>
       </c>
@@ -20114,7 +20115,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>235</v>
       </c>
@@ -20205,7 +20206,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>237</v>
       </c>
@@ -20255,7 +20256,7 @@
         <v>2132</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>238</v>
       </c>
@@ -20305,7 +20306,7 @@
         <v>2126</v>
       </c>
     </row>
-    <row r="257" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>239</v>
       </c>
@@ -20355,7 +20356,7 @@
         <v>2216</v>
       </c>
     </row>
-    <row r="258" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>240</v>
       </c>
@@ -20405,7 +20406,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>241</v>
       </c>
@@ -20455,7 +20456,7 @@
         <v>2224</v>
       </c>
     </row>
-    <row r="260" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>242</v>
       </c>
@@ -20505,7 +20506,7 @@
         <v>2128</v>
       </c>
     </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>243</v>
       </c>
@@ -20552,7 +20553,7 @@
         <v>2221</v>
       </c>
     </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>244</v>
       </c>
@@ -20646,7 +20647,7 @@
         <v>2229</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>246</v>
       </c>
@@ -20696,7 +20697,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>247</v>
       </c>
@@ -20743,7 +20744,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="266" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>248</v>
       </c>
@@ -20793,7 +20794,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="267" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>249</v>
       </c>
@@ -20843,7 +20844,7 @@
         <v>2230</v>
       </c>
     </row>
-    <row r="268" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>250</v>
       </c>
@@ -20893,7 +20894,7 @@
         <v>2190</v>
       </c>
     </row>
-    <row r="269" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>252</v>
       </c>
@@ -20943,7 +20944,7 @@
         <v>2113</v>
       </c>
     </row>
-    <row r="270" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>253</v>
       </c>
@@ -21037,7 +21038,7 @@
         <v>2128</v>
       </c>
     </row>
-    <row r="272" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>255</v>
       </c>
@@ -21084,7 +21085,7 @@
         <v>2204</v>
       </c>
     </row>
-    <row r="273" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>256</v>
       </c>
@@ -21134,7 +21135,7 @@
         <v>2123</v>
       </c>
     </row>
-    <row r="274" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>257</v>
       </c>
@@ -21184,7 +21185,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="275" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>310</v>
       </c>
@@ -21228,7 +21229,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>258</v>
       </c>
@@ -21275,7 +21276,7 @@
         <v>2130</v>
       </c>
     </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>285</v>
       </c>
@@ -21319,7 +21320,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="278" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>226</v>
       </c>
@@ -21369,7 +21370,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>259</v>
       </c>
@@ -21419,7 +21420,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>316</v>
       </c>
@@ -21463,7 +21464,7 @@
         <v>2239</v>
       </c>
     </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>260</v>
       </c>
@@ -21513,7 +21514,7 @@
         <v>2114</v>
       </c>
     </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>315</v>
       </c>
@@ -21557,7 +21558,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="283" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>261</v>
       </c>
@@ -21607,7 +21608,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="284" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>262</v>
       </c>
@@ -21657,7 +21658,7 @@
         <v>2239</v>
       </c>
     </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>263</v>
       </c>
@@ -21707,7 +21708,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="286" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>317</v>
       </c>
@@ -21751,7 +21752,7 @@
         <v>2245</v>
       </c>
     </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>264</v>
       </c>
@@ -21801,7 +21802,7 @@
         <v>2246</v>
       </c>
     </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>265</v>
       </c>
@@ -21851,7 +21852,7 @@
         <v>2247</v>
       </c>
     </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>266</v>
       </c>
@@ -21901,7 +21902,7 @@
         <v>2125</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>267</v>
       </c>
@@ -21951,7 +21952,7 @@
         <v>2249</v>
       </c>
     </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>269</v>
       </c>
@@ -21998,7 +21999,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>270</v>
       </c>
@@ -22048,7 +22049,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="293" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>271</v>
       </c>
@@ -22098,7 +22099,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="294" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>272</v>
       </c>
@@ -22192,7 +22193,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>274</v>
       </c>
@@ -22242,7 +22243,7 @@
         <v>2108</v>
       </c>
     </row>
-    <row r="297" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>275</v>
       </c>
@@ -22292,7 +22293,7 @@
         <v>2164</v>
       </c>
     </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>276</v>
       </c>
@@ -22342,7 +22343,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>277</v>
       </c>
@@ -22392,7 +22393,7 @@
         <v>2251</v>
       </c>
     </row>
-    <row r="300" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>278</v>
       </c>
@@ -22439,7 +22440,7 @@
         <v>2168</v>
       </c>
     </row>
-    <row r="301" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>309</v>
       </c>
@@ -22484,6 +22485,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="L1:L301" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="other"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O301">
     <sortCondition ref="B2:B301"/>
   </sortState>

</xml_diff>